<commit_message>
haciendo interactive dashboards with PowerBI
</commit_message>
<xml_diff>
--- a/Control_Ventas.xlsx
+++ b/Control_Ventas.xlsx
@@ -1,20 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data D Codes Leandro\PowerBI\MiniProyecto-Administrativo-con-excel-o-data-entry\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A8B7D4C-2DD6-4DA2-A6DE-02C4820262FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ventas" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="61">
   <si>
     <t>Fecha</t>
   </si>
@@ -202,11 +221,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -244,28 +263,36 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:F51" totalsRowShown="0">
-  <autoFilter ref="A1:F51"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:F51" totalsRowShown="0">
+  <autoFilter ref="A1:F51" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="6">
-    <tableColumn id="1" name="Fecha"/>
-    <tableColumn id="2" name="Producto"/>
-    <tableColumn id="3" name="Cliente"/>
-    <tableColumn id="4" name="Cantidad"/>
-    <tableColumn id="5" name="Precio"/>
-    <tableColumn id="6" name="Total"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Fecha"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Producto"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Cliente"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Cantidad"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Precio"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Total"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -303,7 +330,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -337,6 +364,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -371,9 +399,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -546,11 +575,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G51"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F51"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -570,7 +599,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>46082</v>
       </c>
@@ -589,12 +618,8 @@
       <c r="F2">
         <v>50</v>
       </c>
-      <c r="G2">
-        <f>IF(D2&gt;10,"Revisar","OK")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>46083</v>
       </c>
@@ -614,7 +639,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>46084</v>
       </c>
@@ -634,7 +659,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>46085</v>
       </c>
@@ -654,7 +679,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>46086</v>
       </c>
@@ -674,7 +699,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>46087</v>
       </c>
@@ -694,7 +719,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>46088</v>
       </c>
@@ -714,7 +739,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>46089</v>
       </c>
@@ -734,7 +759,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>46090</v>
       </c>
@@ -754,7 +779,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>46091</v>
       </c>
@@ -774,7 +799,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>46092</v>
       </c>
@@ -794,7 +819,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>46093</v>
       </c>
@@ -814,7 +839,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>46094</v>
       </c>
@@ -834,7 +859,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>46095</v>
       </c>
@@ -854,7 +879,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>46096</v>
       </c>
@@ -874,7 +899,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>46097</v>
       </c>
@@ -894,7 +919,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>46098</v>
       </c>
@@ -914,7 +939,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>46099</v>
       </c>
@@ -934,7 +959,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>46100</v>
       </c>
@@ -954,7 +979,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>46101</v>
       </c>
@@ -974,7 +999,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>46102</v>
       </c>
@@ -994,7 +1019,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>46103</v>
       </c>
@@ -1014,7 +1039,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>46104</v>
       </c>
@@ -1034,7 +1059,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>46105</v>
       </c>
@@ -1054,7 +1079,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>46106</v>
       </c>
@@ -1074,7 +1099,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>46107</v>
       </c>
@@ -1094,7 +1119,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>46108</v>
       </c>
@@ -1114,7 +1139,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="29" spans="1:6">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>46109</v>
       </c>
@@ -1134,7 +1159,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="30" spans="1:6">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>46110</v>
       </c>
@@ -1154,7 +1179,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="31" spans="1:6">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>46111</v>
       </c>
@@ -1174,7 +1199,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="32" spans="1:6">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>46112</v>
       </c>
@@ -1194,7 +1219,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="33" spans="1:6">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
         <v>46113</v>
       </c>
@@ -1214,7 +1239,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="34" spans="1:6">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="1">
         <v>46114</v>
       </c>
@@ -1234,7 +1259,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="35" spans="1:6">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="1">
         <v>46115</v>
       </c>
@@ -1254,7 +1279,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="36" spans="1:6">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="1">
         <v>46116</v>
       </c>
@@ -1274,7 +1299,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="37" spans="1:6">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="1">
         <v>46117</v>
       </c>
@@ -1294,7 +1319,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="38" spans="1:6">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="1">
         <v>46118</v>
       </c>
@@ -1314,7 +1339,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="39" spans="1:6">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="1">
         <v>46119</v>
       </c>
@@ -1334,7 +1359,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="40" spans="1:6">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="1">
         <v>46120</v>
       </c>
@@ -1354,7 +1379,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="41" spans="1:6">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="1">
         <v>46121</v>
       </c>
@@ -1374,7 +1399,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="42" spans="1:6">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="1">
         <v>46122</v>
       </c>
@@ -1394,7 +1419,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="43" spans="1:6">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" s="1">
         <v>46123</v>
       </c>
@@ -1414,7 +1439,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="44" spans="1:6">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" s="1">
         <v>46124</v>
       </c>
@@ -1434,7 +1459,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="45" spans="1:6">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" s="1">
         <v>46125</v>
       </c>
@@ -1454,7 +1479,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="46" spans="1:6">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" s="1">
         <v>46126</v>
       </c>
@@ -1474,7 +1499,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="47" spans="1:6">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" s="1">
         <v>46127</v>
       </c>
@@ -1494,7 +1519,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="48" spans="1:6">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" s="1">
         <v>46128</v>
       </c>
@@ -1514,7 +1539,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="49" spans="1:6">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" s="1">
         <v>46129</v>
       </c>
@@ -1534,7 +1559,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="50" spans="1:6">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="1">
         <v>46130</v>
       </c>
@@ -1554,7 +1579,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="51" spans="1:6">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" s="1">
         <v>46131</v>
       </c>

</xml_diff>